<commit_message>
Add PECH logos and watermarks to all 227 documents (MD, PDF, DOCX, XLSX)
- Added pech_logo_horizontal.svg to all 65 markdown document headers
- Added watermark dividers ("PECH GROUP HOLDINGS LTD" in subtle styling) throughout documents
- Added branded watermark footer with icon, repeating company name, and confidential line
- Regenerated all 59 PDFs with logo header, branded CSS, watermark background, and footer
- Regenerated all 60 DOCX files with logo in header, colored dividers, and watermark footer
- Updated all 40 XLSX files with logo image, PECH branded header rows, and watermark text
- Generated PNG versions of logos for DOCX/XLSX embedding

https://claude.ai/code/session_014AKpynNrHyqLfWAM6MLBvL
</commit_message>
<xml_diff>
--- a/PECH_CANDIDATE_APPLICATION_FORM.xlsx
+++ b/PECH_CANDIDATE_APPLICATION_FORM.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,8 +85,36 @@
       <color rgb="00999999"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000099CC"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00F5A623"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00888888"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00E8F4F8"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="7"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -117,8 +145,14 @@
         <bgColor rgb="000099CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5A623"/>
+        <bgColor rgb="00F5A623"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -140,11 +174,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -179,6 +257,29 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -255,6 +356,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="628650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -546,7 +677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E176"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -556,118 +687,121 @@
     <col width="25" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>PECH GROUP HOLDINGS LTD</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Technology &amp; Infrastructure Enablers for People</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="4" customHeight="1">
+      <c r="A3" s="15" t="n"/>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
+      <c r="E3" s="15" t="n"/>
+      <c r="F3" s="15" t="n"/>
+      <c r="G3" s="15" t="n"/>
+      <c r="H3" s="15" t="n"/>
+    </row>
+    <row r="4" ht="2" customHeight="1">
+      <c r="A4" s="16" t="n"/>
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="16" t="n"/>
+      <c r="H4" s="16" t="n"/>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Lagos, Nigeria  |  pechgroupholdings.tech  |  Confidential</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="8" customHeight="1"/>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>PECH GROUP HOLDINGS LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>CANDIDATE APPLICATION FORM — CONFIDENTIAL</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Lagos, Nigeria | pechgroupholdings.tech | Ref: PECH-HR-CAF-2026-____</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>SECTION 1: PERSONAL INFORMATION</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Surname / Last Name</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>First Name</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Middle Name</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Date of Birth (DD/MM/YYYY)</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Gender</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Marital Status</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Nationality</t>
+          <t>Surname / Last Name</t>
         </is>
       </c>
       <c r="C12" s="6" t="n"/>
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="19" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>State of Origin</t>
+          <t>First Name</t>
         </is>
       </c>
       <c r="C13" s="6" t="n"/>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="19" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Local Government Area (LGA)</t>
+          <t>Middle Name</t>
         </is>
       </c>
       <c r="C14" s="6" t="n"/>
+      <c r="D14" s="18" t="n"/>
+      <c r="E14" s="19" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Phone Number (Primary)</t>
+          <t>Date of Birth (DD/MM/YYYY)</t>
         </is>
       </c>
       <c r="C15" s="6" t="n"/>
+      <c r="D15" s="18" t="n"/>
+      <c r="E15" s="19" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Phone Number (Secondary)</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="C16" s="6" t="n"/>
@@ -675,7 +809,7 @@
     <row r="17">
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>WhatsApp Number</t>
+          <t>Marital Status</t>
         </is>
       </c>
       <c r="C17" s="6" t="n"/>
@@ -683,202 +817,237 @@
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Email Address</t>
+          <t>Nationality</t>
         </is>
       </c>
       <c r="C18" s="6" t="n"/>
+      <c r="D18" s="18" t="n"/>
+      <c r="E18" s="19" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Residential Address</t>
+          <t>State of Origin</t>
         </is>
       </c>
       <c r="C19" s="6" t="n"/>
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="19" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>Local Government Area (LGA)</t>
         </is>
       </c>
       <c r="C20" s="6" t="n"/>
+      <c r="D20" s="18" t="n"/>
+      <c r="E20" s="19" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Phone Number (Primary)</t>
         </is>
       </c>
       <c r="C21" s="6" t="n"/>
+      <c r="D21" s="18" t="n"/>
+      <c r="E21" s="19" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>NIN (National ID Number)</t>
+          <t>Phone Number (Secondary)</t>
         </is>
       </c>
       <c r="C22" s="6" t="n"/>
+      <c r="D22" s="18" t="n"/>
+      <c r="E22" s="19" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp Number</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="18" t="n"/>
+      <c r="E23" s="19" t="n"/>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>SECTION 2: POSITION APPLIED FOR</t>
-        </is>
-      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Email Address</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="18" t="n"/>
+      <c r="E24" s="19" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Position / Job Title</t>
+          <t>Residential Address</t>
         </is>
       </c>
       <c r="C25" s="6" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="19" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Role ID (if known)</t>
+          <t>City</t>
         </is>
       </c>
       <c r="C26" s="6" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="19" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Department</t>
+          <t>State</t>
         </is>
       </c>
       <c r="C27" s="6" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="19" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Employment Type</t>
+          <t>NIN (National ID Number)</t>
         </is>
       </c>
       <c r="C28" s="6" t="n"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Expected Monthly Salary (NGN)</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="n"/>
-    </row>
+      <c r="D28" s="18" t="n"/>
+      <c r="E28" s="19" t="n"/>
+    </row>
+    <row r="29"/>
     <row r="30">
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Available Start Date</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="n"/>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>SECTION 2: POSITION APPLIED FOR</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Notice Period (if employed)</t>
+          <t>Position / Job Title</t>
         </is>
       </c>
       <c r="C31" s="6" t="n"/>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="19" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="5" t="inlineStr">
         <is>
+          <t>Role ID (if known)</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n"/>
+      <c r="D32" s="18" t="n"/>
+      <c r="E32" s="19" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="n"/>
+    </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Employment Type</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Expected Monthly Salary (NGN)</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="18" t="n"/>
+      <c r="E35" s="19" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Available Start Date</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="18" t="n"/>
+      <c r="E36" s="19" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Notice Period (if employed)</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="18" t="n"/>
+      <c r="E37" s="19" t="n"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="5" t="inlineStr">
+        <is>
           <t>How did you hear about us?</t>
         </is>
       </c>
-      <c r="C32" s="6" t="n"/>
-    </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="C38" s="6" t="n"/>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>SECTION 3: EDUCATIONAL BACKGROUND</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="7" t="inlineStr">
+    <row r="41">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>List all qualifications starting from the most recent</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" s="8" t="inlineStr">
+    <row r="42">
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
         <is>
           <t>Qualification</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="D42" s="8" t="inlineStr">
         <is>
           <t>Course of Study</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E42" s="8" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="6" t="n"/>
-      <c r="D37" s="6" t="n"/>
-      <c r="E37" s="6" t="n"/>
-    </row>
-    <row r="38">
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="6" t="n"/>
-      <c r="E38" s="6" t="n"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="6" t="n"/>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="6" t="n"/>
-    </row>
-    <row r="40">
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="6" t="n"/>
-      <c r="D40" s="6" t="n"/>
-      <c r="E40" s="6" t="n"/>
-    </row>
-    <row r="42">
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>Professional Certifications</t>
-        </is>
-      </c>
-    </row>
     <row r="43">
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>Certification Name</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>Issuing Body</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Year Obtained</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Certificate No.</t>
-        </is>
-      </c>
+      <c r="B43" s="6" t="n"/>
+      <c r="C43" s="6" t="n"/>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="B44" s="6" t="n"/>
@@ -898,324 +1067,389 @@
       <c r="D46" s="6" t="n"/>
       <c r="E46" s="6" t="n"/>
     </row>
+    <row r="47"/>
     <row r="48" ht="28" customHeight="1">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Professional Certifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Certification Name</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Issuing Body</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Year Obtained</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Certificate No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="6" t="n"/>
+      <c r="C50" s="6" t="n"/>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" s="6" t="n"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="6" t="n"/>
+      <c r="C51" s="6" t="n"/>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="6" t="n"/>
+      <c r="C52" s="6" t="n"/>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" s="6" t="n"/>
+    </row>
+    <row r="53"/>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>SECTION 4: WORK EXPERIENCE</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="7" t="inlineStr">
+    <row r="55">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>List your last 3 positions (most recent first). Write N/A if no experience.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" s="9" t="inlineStr">
+    <row r="56"/>
+    <row r="57">
+      <c r="B57" s="9" t="inlineStr">
         <is>
           <t>Position 1 (Most Recent)</t>
         </is>
       </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Company / Organisation</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="n"/>
-    </row>
-    <row r="53">
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>Your Job Title</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="n"/>
-    </row>
-    <row r="54">
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>Employment Type</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="n"/>
-    </row>
-    <row r="55">
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="n"/>
-    </row>
-    <row r="56">
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>End Date (or 'Present')</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="n"/>
-    </row>
-    <row r="57">
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>Monthly Salary (NGN)</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Supervisor Name &amp; Phone</t>
+          <t>Company / Organisation</t>
         </is>
       </c>
       <c r="C58" s="6" t="n"/>
+      <c r="D58" s="18" t="n"/>
+      <c r="E58" s="19" t="n"/>
     </row>
     <row r="59">
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Reason for Leaving</t>
+          <t>Your Job Title</t>
         </is>
       </c>
       <c r="C59" s="6" t="n"/>
+      <c r="D59" s="18" t="n"/>
+      <c r="E59" s="19" t="n"/>
     </row>
     <row r="60">
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Key Responsibilities</t>
+          <t>Employment Type</t>
         </is>
       </c>
       <c r="C60" s="6" t="n"/>
     </row>
+    <row r="61">
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="n"/>
+      <c r="D61" s="18" t="n"/>
+      <c r="E61" s="19" t="n"/>
+    </row>
     <row r="62">
-      <c r="B62" s="9" t="inlineStr">
-        <is>
-          <t>Position 2</t>
-        </is>
-      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>End Date (or 'Present')</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="n"/>
+      <c r="D62" s="18" t="n"/>
+      <c r="E62" s="19" t="n"/>
     </row>
     <row r="63">
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Company / Organisation</t>
+          <t>Monthly Salary (NGN)</t>
         </is>
       </c>
       <c r="C63" s="6" t="n"/>
+      <c r="D63" s="18" t="n"/>
+      <c r="E63" s="19" t="n"/>
     </row>
     <row r="64">
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Your Job Title</t>
+          <t>Supervisor Name &amp; Phone</t>
         </is>
       </c>
       <c r="C64" s="6" t="n"/>
+      <c r="D64" s="18" t="n"/>
+      <c r="E64" s="19" t="n"/>
     </row>
     <row r="65">
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Employment Type</t>
+          <t>Reason for Leaving</t>
         </is>
       </c>
       <c r="C65" s="6" t="n"/>
+      <c r="D65" s="18" t="n"/>
+      <c r="E65" s="19" t="n"/>
     </row>
     <row r="66">
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>Key Responsibilities</t>
         </is>
       </c>
       <c r="C66" s="6" t="n"/>
-    </row>
-    <row r="67">
-      <c r="B67" s="5" t="inlineStr">
-        <is>
-          <t>End Date (or 'Present')</t>
-        </is>
-      </c>
-      <c r="C67" s="6" t="n"/>
-    </row>
+      <c r="D66" s="18" t="n"/>
+      <c r="E66" s="19" t="n"/>
+    </row>
+    <row r="67"/>
     <row r="68">
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>Monthly Salary (NGN)</t>
-        </is>
-      </c>
-      <c r="C68" s="6" t="n"/>
+      <c r="B68" s="9" t="inlineStr">
+        <is>
+          <t>Position 2</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Supervisor Name &amp; Phone</t>
+          <t>Company / Organisation</t>
         </is>
       </c>
       <c r="C69" s="6" t="n"/>
+      <c r="D69" s="18" t="n"/>
+      <c r="E69" s="19" t="n"/>
     </row>
     <row r="70">
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Reason for Leaving</t>
+          <t>Your Job Title</t>
         </is>
       </c>
       <c r="C70" s="6" t="n"/>
+      <c r="D70" s="18" t="n"/>
+      <c r="E70" s="19" t="n"/>
     </row>
     <row r="71">
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>Key Responsibilities</t>
+          <t>Employment Type</t>
         </is>
       </c>
       <c r="C71" s="6" t="n"/>
     </row>
+    <row r="72">
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="n"/>
+      <c r="D72" s="18" t="n"/>
+      <c r="E72" s="19" t="n"/>
+    </row>
     <row r="73">
-      <c r="B73" s="9" t="inlineStr">
-        <is>
-          <t>Position 3</t>
-        </is>
-      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>End Date (or 'Present')</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="n"/>
+      <c r="D73" s="18" t="n"/>
+      <c r="E73" s="19" t="n"/>
     </row>
     <row r="74">
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Company / Organisation</t>
+          <t>Monthly Salary (NGN)</t>
         </is>
       </c>
       <c r="C74" s="6" t="n"/>
+      <c r="D74" s="18" t="n"/>
+      <c r="E74" s="19" t="n"/>
     </row>
     <row r="75">
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Your Job Title</t>
+          <t>Supervisor Name &amp; Phone</t>
         </is>
       </c>
       <c r="C75" s="6" t="n"/>
+      <c r="D75" s="18" t="n"/>
+      <c r="E75" s="19" t="n"/>
     </row>
     <row r="76">
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Employment Type</t>
+          <t>Reason for Leaving</t>
         </is>
       </c>
       <c r="C76" s="6" t="n"/>
+      <c r="D76" s="18" t="n"/>
+      <c r="E76" s="19" t="n"/>
     </row>
     <row r="77">
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>Start Date</t>
+          <t>Key Responsibilities</t>
         </is>
       </c>
       <c r="C77" s="6" t="n"/>
-    </row>
-    <row r="78">
-      <c r="B78" s="5" t="inlineStr">
-        <is>
-          <t>End Date (or 'Present')</t>
-        </is>
-      </c>
-      <c r="C78" s="6" t="n"/>
-    </row>
+      <c r="D77" s="18" t="n"/>
+      <c r="E77" s="19" t="n"/>
+    </row>
+    <row r="78"/>
     <row r="79">
-      <c r="B79" s="5" t="inlineStr">
-        <is>
-          <t>Monthly Salary (NGN)</t>
-        </is>
-      </c>
-      <c r="C79" s="6" t="n"/>
+      <c r="B79" s="9" t="inlineStr">
+        <is>
+          <t>Position 3</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Supervisor Name &amp; Phone</t>
+          <t>Company / Organisation</t>
         </is>
       </c>
       <c r="C80" s="6" t="n"/>
+      <c r="D80" s="18" t="n"/>
+      <c r="E80" s="19" t="n"/>
     </row>
     <row r="81">
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>Reason for Leaving</t>
+          <t>Your Job Title</t>
         </is>
       </c>
       <c r="C81" s="6" t="n"/>
+      <c r="D81" s="18" t="n"/>
+      <c r="E81" s="19" t="n"/>
     </row>
     <row r="82">
       <c r="B82" s="5" t="inlineStr">
         <is>
+          <t>Employment Type</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="n"/>
+    </row>
+    <row r="83">
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="n"/>
+      <c r="D83" s="18" t="n"/>
+      <c r="E83" s="19" t="n"/>
+    </row>
+    <row r="84" ht="28" customHeight="1">
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>End Date (or 'Present')</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="n"/>
+      <c r="D84" s="18" t="n"/>
+      <c r="E84" s="19" t="n"/>
+    </row>
+    <row r="85">
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Monthly Salary (NGN)</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="n"/>
+      <c r="D85" s="18" t="n"/>
+      <c r="E85" s="19" t="n"/>
+    </row>
+    <row r="86">
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Supervisor Name &amp; Phone</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="n"/>
+      <c r="D86" s="18" t="n"/>
+      <c r="E86" s="19" t="n"/>
+    </row>
+    <row r="87">
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Reason for Leaving</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="n"/>
+      <c r="D87" s="18" t="n"/>
+      <c r="E87" s="19" t="n"/>
+    </row>
+    <row r="88">
+      <c r="B88" s="5" t="inlineStr">
+        <is>
           <t>Key Responsibilities</t>
         </is>
       </c>
-      <c r="C82" s="6" t="n"/>
-    </row>
-    <row r="84" ht="28" customHeight="1">
-      <c r="A84" s="4" t="inlineStr">
+      <c r="C88" s="6" t="n"/>
+      <c r="D88" s="18" t="n"/>
+      <c r="E88" s="19" t="n"/>
+    </row>
+    <row r="89"/>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
         <is>
           <t>SECTION 5: TECHNICAL SKILLS &amp; COMPETENCIES</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="B85" s="7" t="inlineStr">
+    <row r="91">
+      <c r="B91" s="7" t="inlineStr">
         <is>
           <t>For technical roles. Non-technical applicants may skip to General Competencies below.</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="B86" s="8" t="inlineStr">
+    <row r="92">
+      <c r="B92" s="8" t="inlineStr">
         <is>
           <t>Skill / Technology</t>
         </is>
       </c>
-      <c r="C86" s="8" t="inlineStr">
+      <c r="C92" s="8" t="inlineStr">
         <is>
           <t>Proficiency Level</t>
         </is>
       </c>
-      <c r="D86" s="8" t="inlineStr">
+      <c r="D92" s="8" t="inlineStr">
         <is>
           <t>Years of Experience</t>
         </is>
       </c>
-      <c r="E86" s="8" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="B87" s="10" t="n"/>
-      <c r="C87" s="10" t="inlineStr"/>
-      <c r="D87" s="10" t="n"/>
-      <c r="E87" s="10" t="n"/>
-    </row>
-    <row r="88">
-      <c r="B88" s="10" t="n"/>
-      <c r="C88" s="10" t="inlineStr"/>
-      <c r="D88" s="10" t="n"/>
-      <c r="E88" s="10" t="n"/>
-    </row>
-    <row r="89">
-      <c r="B89" s="10" t="n"/>
-      <c r="C89" s="10" t="inlineStr"/>
-      <c r="D89" s="10" t="n"/>
-      <c r="E89" s="10" t="n"/>
-    </row>
-    <row r="90">
-      <c r="B90" s="10" t="n"/>
-      <c r="C90" s="10" t="inlineStr"/>
-      <c r="D90" s="10" t="n"/>
-      <c r="E90" s="10" t="n"/>
-    </row>
-    <row r="91">
-      <c r="B91" s="10" t="n"/>
-      <c r="C91" s="10" t="inlineStr"/>
-      <c r="D91" s="10" t="n"/>
-      <c r="E91" s="10" t="n"/>
-    </row>
-    <row r="92">
-      <c r="B92" s="10" t="n"/>
-      <c r="C92" s="10" t="inlineStr"/>
-      <c r="D92" s="10" t="n"/>
-      <c r="E92" s="10" t="n"/>
+      <c r="E92" s="8" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="B93" s="10" t="n"/>
@@ -1229,289 +1463,340 @@
       <c r="D94" s="10" t="n"/>
       <c r="E94" s="10" t="n"/>
     </row>
+    <row r="95">
+      <c r="B95" s="10" t="n"/>
+      <c r="C95" s="10" t="inlineStr"/>
+      <c r="D95" s="10" t="n"/>
+      <c r="E95" s="10" t="n"/>
+    </row>
     <row r="96">
-      <c r="B96" s="5" t="inlineStr">
-        <is>
-          <t>Portfolio Website URL</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="n"/>
+      <c r="B96" s="10" t="n"/>
+      <c r="C96" s="10" t="inlineStr"/>
+      <c r="D96" s="10" t="n"/>
+      <c r="E96" s="10" t="n"/>
     </row>
     <row r="97">
-      <c r="B97" s="5" t="inlineStr">
-        <is>
-          <t>GitHub Profile URL</t>
-        </is>
-      </c>
-      <c r="C97" s="6" t="n"/>
+      <c r="B97" s="10" t="n"/>
+      <c r="C97" s="10" t="inlineStr"/>
+      <c r="D97" s="10" t="n"/>
+      <c r="E97" s="10" t="n"/>
     </row>
     <row r="98">
-      <c r="B98" s="5" t="inlineStr">
-        <is>
-          <t>LinkedIn Profile URL</t>
-        </is>
-      </c>
-      <c r="C98" s="6" t="n"/>
+      <c r="B98" s="10" t="n"/>
+      <c r="C98" s="10" t="inlineStr"/>
+      <c r="D98" s="10" t="n"/>
+      <c r="E98" s="10" t="n"/>
+    </row>
+    <row r="99">
+      <c r="B99" s="10" t="n"/>
+      <c r="C99" s="10" t="inlineStr"/>
+      <c r="D99" s="10" t="n"/>
+      <c r="E99" s="10" t="n"/>
     </row>
     <row r="100" ht="28" customHeight="1">
-      <c r="A100" s="4" t="inlineStr">
-        <is>
-          <t>SECTION 6: REFERENCES (Minimum 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="B101" s="9" t="inlineStr">
-        <is>
-          <t>Reference 1</t>
-        </is>
-      </c>
-    </row>
+      <c r="B100" s="10" t="n"/>
+      <c r="C100" s="10" t="inlineStr"/>
+      <c r="D100" s="10" t="n"/>
+      <c r="E100" s="10" t="n"/>
+    </row>
+    <row r="101"/>
     <row r="102">
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>Full Name</t>
+          <t>Portfolio Website URL</t>
         </is>
       </c>
       <c r="C102" s="6" t="n"/>
+      <c r="D102" s="18" t="n"/>
+      <c r="E102" s="19" t="n"/>
     </row>
     <row r="103">
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>Relationship</t>
+          <t>GitHub Profile URL</t>
         </is>
       </c>
       <c r="C103" s="6" t="n"/>
+      <c r="D103" s="18" t="n"/>
+      <c r="E103" s="19" t="n"/>
     </row>
     <row r="104">
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>Organisation &amp; Position</t>
+          <t>LinkedIn Profile URL</t>
         </is>
       </c>
       <c r="C104" s="6" t="n"/>
-    </row>
-    <row r="105">
-      <c r="B105" s="5" t="inlineStr">
-        <is>
-          <t>Phone Number</t>
-        </is>
-      </c>
-      <c r="C105" s="6" t="n"/>
-    </row>
+      <c r="D104" s="18" t="n"/>
+      <c r="E104" s="19" t="n"/>
+    </row>
+    <row r="105"/>
     <row r="106">
-      <c r="B106" s="5" t="inlineStr">
-        <is>
-          <t>Email Address</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="n"/>
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>SECTION 6: REFERENCES (Minimum 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="9" t="inlineStr">
+        <is>
+          <t>Reference 1</t>
+        </is>
+      </c>
     </row>
     <row r="108">
-      <c r="B108" s="9" t="inlineStr">
-        <is>
-          <t>Reference 2</t>
-        </is>
-      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>Full Name</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="n"/>
+      <c r="D108" s="18" t="n"/>
+      <c r="E108" s="19" t="n"/>
     </row>
     <row r="109">
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>Full Name</t>
+          <t>Relationship</t>
         </is>
       </c>
       <c r="C109" s="6" t="n"/>
+      <c r="D109" s="18" t="n"/>
+      <c r="E109" s="19" t="n"/>
     </row>
     <row r="110">
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>Relationship</t>
+          <t>Organisation &amp; Position</t>
         </is>
       </c>
       <c r="C110" s="6" t="n"/>
+      <c r="D110" s="18" t="n"/>
+      <c r="E110" s="19" t="n"/>
     </row>
     <row r="111">
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>Organisation &amp; Position</t>
+          <t>Phone Number</t>
         </is>
       </c>
       <c r="C111" s="6" t="n"/>
+      <c r="D111" s="18" t="n"/>
+      <c r="E111" s="19" t="n"/>
     </row>
     <row r="112">
       <c r="B112" s="5" t="inlineStr">
         <is>
+          <t>Email Address</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="n"/>
+      <c r="D112" s="18" t="n"/>
+      <c r="E112" s="19" t="n"/>
+    </row>
+    <row r="113"/>
+    <row r="114">
+      <c r="B114" s="9" t="inlineStr">
+        <is>
+          <t>Reference 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>Full Name</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="n"/>
+      <c r="D115" s="18" t="n"/>
+      <c r="E115" s="19" t="n"/>
+    </row>
+    <row r="116" ht="28" customHeight="1">
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>Relationship</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="n"/>
+      <c r="D116" s="18" t="n"/>
+      <c r="E116" s="19" t="n"/>
+    </row>
+    <row r="117">
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Organisation &amp; Position</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="n"/>
+      <c r="D117" s="18" t="n"/>
+      <c r="E117" s="19" t="n"/>
+    </row>
+    <row r="118">
+      <c r="B118" s="5" t="inlineStr">
+        <is>
           <t>Phone Number</t>
         </is>
       </c>
-      <c r="C112" s="6" t="n"/>
-    </row>
-    <row r="113">
-      <c r="B113" s="5" t="inlineStr">
-        <is>
-          <t>Email Address</t>
-        </is>
-      </c>
-      <c r="C113" s="6" t="n"/>
-    </row>
-    <row r="116" ht="28" customHeight="1">
-      <c r="A116" s="4" t="inlineStr">
-        <is>
-          <t>SECTION 7: GUARANTOR INFORMATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="B117" s="7" t="inlineStr">
-        <is>
-          <t>Two guarantors required. Full Guarantor Forms will be completed upon offer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="B118" s="9" t="inlineStr">
-        <is>
-          <t>Guarantor 1</t>
-        </is>
-      </c>
+      <c r="C118" s="6" t="n"/>
+      <c r="D118" s="18" t="n"/>
+      <c r="E118" s="19" t="n"/>
     </row>
     <row r="119">
       <c r="B119" s="5" t="inlineStr">
         <is>
+          <t>Email Address</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="n"/>
+      <c r="D119" s="18" t="n"/>
+      <c r="E119" s="19" t="n"/>
+    </row>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>SECTION 7: GUARANTOR INFORMATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" s="7" t="inlineStr">
+        <is>
+          <t>Two guarantors required. Full Guarantor Forms will be completed upon offer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" s="9" t="inlineStr">
+        <is>
+          <t>Guarantor 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" s="5" t="inlineStr">
+        <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="C119" s="6" t="n"/>
-    </row>
-    <row r="120">
-      <c r="B120" s="5" t="inlineStr">
-        <is>
-          <t>Occupation</t>
-        </is>
-      </c>
-      <c r="C120" s="6" t="n"/>
-    </row>
-    <row r="121">
-      <c r="B121" s="5" t="inlineStr">
-        <is>
-          <t>Organisation / Employer</t>
-        </is>
-      </c>
-      <c r="C121" s="6" t="n"/>
-    </row>
-    <row r="122">
-      <c r="B122" s="5" t="inlineStr">
-        <is>
-          <t>Phone Number</t>
-        </is>
-      </c>
-      <c r="C122" s="6" t="n"/>
-    </row>
-    <row r="123">
-      <c r="B123" s="5" t="inlineStr">
-        <is>
-          <t>Residential Address</t>
-        </is>
-      </c>
-      <c r="C123" s="6" t="n"/>
-    </row>
-    <row r="125">
-      <c r="B125" s="9" t="inlineStr">
-        <is>
-          <t>Guarantor 2</t>
-        </is>
-      </c>
+      <c r="C125" s="6" t="n"/>
+      <c r="D125" s="18" t="n"/>
+      <c r="E125" s="19" t="n"/>
     </row>
     <row r="126">
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>Full Name</t>
+          <t>Occupation</t>
         </is>
       </c>
       <c r="C126" s="6" t="n"/>
+      <c r="D126" s="18" t="n"/>
+      <c r="E126" s="19" t="n"/>
     </row>
     <row r="127">
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>Occupation</t>
+          <t>Organisation / Employer</t>
         </is>
       </c>
       <c r="C127" s="6" t="n"/>
+      <c r="D127" s="18" t="n"/>
+      <c r="E127" s="19" t="n"/>
     </row>
     <row r="128">
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>Organisation / Employer</t>
+          <t>Phone Number</t>
         </is>
       </c>
       <c r="C128" s="6" t="n"/>
+      <c r="D128" s="18" t="n"/>
+      <c r="E128" s="19" t="n"/>
     </row>
     <row r="129">
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>Phone Number</t>
+          <t>Residential Address</t>
         </is>
       </c>
       <c r="C129" s="6" t="n"/>
-    </row>
-    <row r="130">
-      <c r="B130" s="5" t="inlineStr">
-        <is>
-          <t>Residential Address</t>
-        </is>
-      </c>
-      <c r="C130" s="6" t="n"/>
+      <c r="D129" s="18" t="n"/>
+      <c r="E129" s="19" t="n"/>
+    </row>
+    <row r="130"/>
+    <row r="131">
+      <c r="B131" s="9" t="inlineStr">
+        <is>
+          <t>Guarantor 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>Full Name</t>
+        </is>
+      </c>
+      <c r="C132" s="6" t="n"/>
+      <c r="D132" s="18" t="n"/>
+      <c r="E132" s="19" t="n"/>
     </row>
     <row r="133" ht="28" customHeight="1">
-      <c r="A133" s="4" t="inlineStr">
-        <is>
-          <t>SECTION 8: HEALTH &amp; EMERGENCY INFORMATION</t>
-        </is>
-      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Occupation</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="n"/>
+      <c r="D133" s="18" t="n"/>
+      <c r="E133" s="19" t="n"/>
     </row>
     <row r="134">
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>Blood Group</t>
+          <t>Organisation / Employer</t>
         </is>
       </c>
       <c r="C134" s="6" t="n"/>
+      <c r="D134" s="18" t="n"/>
+      <c r="E134" s="19" t="n"/>
     </row>
     <row r="135">
       <c r="B135" s="5" t="inlineStr">
         <is>
-          <t>Genotype</t>
+          <t>Phone Number</t>
         </is>
       </c>
       <c r="C135" s="6" t="n"/>
+      <c r="D135" s="18" t="n"/>
+      <c r="E135" s="19" t="n"/>
     </row>
     <row r="136">
       <c r="B136" s="5" t="inlineStr">
         <is>
-          <t>Medical Conditions (if any)</t>
+          <t>Residential Address</t>
         </is>
       </c>
       <c r="C136" s="6" t="n"/>
-    </row>
-    <row r="137">
-      <c r="B137" s="5" t="inlineStr">
-        <is>
-          <t>Disability / Accommodation Needed</t>
-        </is>
-      </c>
-      <c r="C137" s="6" t="n"/>
-    </row>
+      <c r="D136" s="18" t="n"/>
+      <c r="E136" s="19" t="n"/>
+    </row>
+    <row r="137"/>
+    <row r="138"/>
     <row r="139">
-      <c r="B139" s="9" t="inlineStr">
-        <is>
-          <t>Emergency Contact</t>
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>SECTION 8: HEALTH &amp; EMERGENCY INFORMATION</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>Full Name</t>
+          <t>Blood Group</t>
         </is>
       </c>
       <c r="C140" s="6" t="n"/>
@@ -1519,7 +1804,7 @@
     <row r="141">
       <c r="B141" s="5" t="inlineStr">
         <is>
-          <t>Relationship</t>
+          <t>Genotype</t>
         </is>
       </c>
       <c r="C141" s="6" t="n"/>
@@ -1527,70 +1812,73 @@
     <row r="142">
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>Phone Number</t>
+          <t>Medical Conditions (if any)</t>
         </is>
       </c>
       <c r="C142" s="6" t="n"/>
-    </row>
-    <row r="144" ht="28" customHeight="1">
-      <c r="A144" s="4" t="inlineStr">
-        <is>
-          <t>SECTION 9: ADDITIONAL DECLARATIONS</t>
-        </is>
-      </c>
-    </row>
+      <c r="D142" s="18" t="n"/>
+      <c r="E142" s="19" t="n"/>
+    </row>
+    <row r="143">
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Disability / Accommodation Needed</t>
+        </is>
+      </c>
+      <c r="C143" s="6" t="n"/>
+      <c r="D143" s="18" t="n"/>
+      <c r="E143" s="19" t="n"/>
+    </row>
+    <row r="144" ht="28" customHeight="1"/>
     <row r="145">
-      <c r="B145" s="5" t="inlineStr">
-        <is>
-          <t>Convicted of a criminal offence?</t>
-        </is>
-      </c>
-      <c r="C145" s="6" t="n"/>
+      <c r="B145" s="9" t="inlineStr">
+        <is>
+          <t>Emergency Contact</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="B146" s="5" t="inlineStr">
         <is>
-          <t>Previously dismissed/terminated?</t>
+          <t>Full Name</t>
         </is>
       </c>
       <c r="C146" s="6" t="n"/>
+      <c r="D146" s="18" t="n"/>
+      <c r="E146" s="19" t="n"/>
     </row>
     <row r="147">
       <c r="B147" s="5" t="inlineStr">
         <is>
-          <t>Ongoing legal proceedings?</t>
+          <t>Relationship</t>
         </is>
       </c>
       <c r="C147" s="6" t="n"/>
+      <c r="D147" s="18" t="n"/>
+      <c r="E147" s="19" t="n"/>
     </row>
     <row r="148">
       <c r="B148" s="5" t="inlineStr">
         <is>
-          <t>Relatives at PECH Group?</t>
+          <t>Phone Number</t>
         </is>
       </c>
       <c r="C148" s="6" t="n"/>
-    </row>
-    <row r="149">
-      <c r="B149" s="5" t="inlineStr">
-        <is>
-          <t>Currently employed elsewhere?</t>
-        </is>
-      </c>
-      <c r="C149" s="6" t="n"/>
-    </row>
+      <c r="D148" s="18" t="n"/>
+      <c r="E148" s="19" t="n"/>
+    </row>
+    <row r="149"/>
     <row r="150">
-      <c r="B150" s="5" t="inlineStr">
-        <is>
-          <t>Willing to relocate in Nigeria?</t>
-        </is>
-      </c>
-      <c r="C150" s="6" t="n"/>
+      <c r="A150" s="4" t="inlineStr">
+        <is>
+          <t>SECTION 9: ADDITIONAL DECLARATIONS</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="B151" s="5" t="inlineStr">
         <is>
-          <t>Willing to travel for work?</t>
+          <t>Convicted of a criminal offence?</t>
         </is>
       </c>
       <c r="C151" s="6" t="n"/>
@@ -1598,7 +1886,7 @@
     <row r="152">
       <c r="B152" s="5" t="inlineStr">
         <is>
-          <t>Valid driver's license?</t>
+          <t>Previously dismissed/terminated?</t>
         </is>
       </c>
       <c r="C152" s="6" t="n"/>
@@ -1606,7 +1894,7 @@
     <row r="153">
       <c r="B153" s="5" t="inlineStr">
         <is>
-          <t>Valid international passport?</t>
+          <t>Ongoing legal proceedings?</t>
         </is>
       </c>
       <c r="C153" s="6" t="n"/>
@@ -1614,7 +1902,7 @@
     <row r="154">
       <c r="B154" s="5" t="inlineStr">
         <is>
-          <t>Authorized to work in Nigeria?</t>
+          <t>Relatives at PECH Group?</t>
         </is>
       </c>
       <c r="C154" s="6" t="n"/>
@@ -1622,128 +1910,238 @@
     <row r="155">
       <c r="B155" s="5" t="inlineStr">
         <is>
-          <t>If 'Yes' to any above, provide details:</t>
+          <t>Currently employed elsewhere?</t>
         </is>
       </c>
       <c r="C155" s="6" t="n"/>
     </row>
+    <row r="156">
+      <c r="B156" s="5" t="inlineStr">
+        <is>
+          <t>Willing to relocate in Nigeria?</t>
+        </is>
+      </c>
+      <c r="C156" s="6" t="n"/>
+    </row>
     <row r="157" ht="28" customHeight="1">
-      <c r="A157" s="4" t="inlineStr">
-        <is>
-          <t>SECTION 10: DECLARATION &amp; CONSENT</t>
-        </is>
-      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>Willing to travel for work?</t>
+        </is>
+      </c>
+      <c r="C157" s="6" t="n"/>
+    </row>
+    <row r="158">
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>Valid driver's license?</t>
+        </is>
+      </c>
+      <c r="C158" s="6" t="n"/>
     </row>
     <row r="159" ht="45" customHeight="1">
-      <c r="B159" s="11" t="inlineStr">
-        <is>
-          <t>I declare that all information in this form is true and accurate. I consent to PECH Group Holdings Ltd processing my data per NDPA 2023. I understand false information may lead to disqualification or termination.</t>
-        </is>
-      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>Valid international passport?</t>
+        </is>
+      </c>
+      <c r="C159" s="6" t="n"/>
+    </row>
+    <row r="160">
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>Authorized to work in Nigeria?</t>
+        </is>
+      </c>
+      <c r="C160" s="6" t="n"/>
     </row>
     <row r="161">
       <c r="B161" s="5" t="inlineStr">
         <is>
-          <t>Applicant's Full Name (Print)</t>
+          <t>If 'Yes' to any above, provide details:</t>
         </is>
       </c>
       <c r="C161" s="6" t="n"/>
-    </row>
-    <row r="162">
-      <c r="B162" s="5" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="C162" s="6" t="n"/>
-    </row>
+      <c r="D161" s="18" t="n"/>
+      <c r="E161" s="19" t="n"/>
+    </row>
+    <row r="162"/>
     <row r="163">
-      <c r="B163" s="5" t="inlineStr">
-        <is>
-          <t>Date (DD/MM/YYYY)</t>
-        </is>
-      </c>
-      <c r="C163" s="6" t="n"/>
-    </row>
+      <c r="A163" s="4" t="inlineStr">
+        <is>
+          <t>SECTION 10: DECLARATION &amp; CONSENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="164"/>
     <row r="165" ht="28" customHeight="1">
-      <c r="A165" s="4" t="inlineStr">
-        <is>
-          <t>SECTION 11: FOR OFFICE USE ONLY</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="B166" s="7" t="inlineStr">
-        <is>
-          <t>To be completed by HR Department only</t>
-        </is>
-      </c>
-    </row>
+      <c r="B165" s="11" t="inlineStr">
+        <is>
+          <t>I declare that all information in this form is true and accurate. I consent to PECH Group Holdings Ltd processing my data per NDPA 2023. I understand false information may lead to disqualification or termination.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166"/>
     <row r="167">
       <c r="B167" s="5" t="inlineStr">
         <is>
-          <t>Application Reference No.</t>
+          <t>Applicant's Full Name (Print)</t>
         </is>
       </c>
       <c r="C167" s="6" t="n"/>
+      <c r="D167" s="18" t="n"/>
+      <c r="E167" s="19" t="n"/>
     </row>
     <row r="168">
       <c r="B168" s="5" t="inlineStr">
         <is>
-          <t>Date Received</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="C168" s="6" t="n"/>
+      <c r="D168" s="18" t="n"/>
+      <c r="E168" s="19" t="n"/>
     </row>
     <row r="169">
       <c r="B169" s="5" t="inlineStr">
         <is>
-          <t>Received By</t>
+          <t>Date (DD/MM/YYYY)</t>
         </is>
       </c>
       <c r="C169" s="6" t="n"/>
-    </row>
-    <row r="170">
-      <c r="B170" s="5" t="inlineStr">
-        <is>
-          <t>Application Complete?</t>
-        </is>
-      </c>
-      <c r="C170" s="6" t="n"/>
-    </row>
+      <c r="D169" s="18" t="n"/>
+      <c r="E169" s="19" t="n"/>
+    </row>
+    <row r="170"/>
     <row r="171">
-      <c r="B171" s="5" t="inlineStr">
-        <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="C171" s="6" t="n"/>
+      <c r="A171" s="4" t="inlineStr">
+        <is>
+          <t>SECTION 11: FOR OFFICE USE ONLY</t>
+        </is>
+      </c>
     </row>
     <row r="172">
-      <c r="B172" s="5" t="inlineStr">
-        <is>
-          <t>Reason for Decision</t>
-        </is>
-      </c>
-      <c r="C172" s="6" t="n"/>
+      <c r="B172" s="7" t="inlineStr">
+        <is>
+          <t>To be completed by HR Department only</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="B173" s="5" t="inlineStr">
         <is>
+          <t>Application Reference No.</t>
+        </is>
+      </c>
+      <c r="C173" s="6" t="n"/>
+      <c r="D173" s="18" t="n"/>
+      <c r="E173" s="19" t="n"/>
+    </row>
+    <row r="174">
+      <c r="B174" s="5" t="inlineStr">
+        <is>
+          <t>Date Received</t>
+        </is>
+      </c>
+      <c r="C174" s="6" t="n"/>
+      <c r="D174" s="18" t="n"/>
+      <c r="E174" s="19" t="n"/>
+    </row>
+    <row r="175">
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>Received By</t>
+        </is>
+      </c>
+      <c r="C175" s="6" t="n"/>
+      <c r="D175" s="18" t="n"/>
+      <c r="E175" s="19" t="n"/>
+    </row>
+    <row r="176">
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>Application Complete?</t>
+        </is>
+      </c>
+      <c r="C176" s="6" t="n"/>
+    </row>
+    <row r="177">
+      <c r="B177" s="5" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C177" s="6" t="n"/>
+    </row>
+    <row r="178">
+      <c r="B178" s="5" t="inlineStr">
+        <is>
+          <t>Reason for Decision</t>
+        </is>
+      </c>
+      <c r="C178" s="6" t="n"/>
+      <c r="D178" s="18" t="n"/>
+      <c r="E178" s="19" t="n"/>
+    </row>
+    <row r="179">
+      <c r="B179" s="5" t="inlineStr">
+        <is>
           <t>Approved By</t>
         </is>
       </c>
-      <c r="C173" s="6" t="n"/>
-    </row>
-    <row r="176">
-      <c r="A176" s="12" t="inlineStr">
+      <c r="C179" s="6" t="n"/>
+      <c r="D179" s="18" t="n"/>
+      <c r="E179" s="19" t="n"/>
+    </row>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182">
+      <c r="A182" s="12" t="inlineStr">
         <is>
           <t>PECH Group Holdings Ltd — Technology &amp; Infrastructure Enablers for People</t>
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" s="20" t="inlineStr">
+        <is>
+          <t>PECH GROUP HOLDINGS LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="20" t="inlineStr">
+        <is>
+          <t>PECH GROUP HOLDINGS LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="20" t="inlineStr">
+        <is>
+          <t>PECH GROUP HOLDINGS LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="21" t="inlineStr">
+        <is>
+          <t>Confidential — PECH Group Holdings Ltd — Lagos, Nigeria — pechgroupholdings.tech</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="15" t="n"/>
+      <c r="B188" s="15" t="n"/>
+      <c r="C188" s="15" t="n"/>
+      <c r="D188" s="15" t="n"/>
+      <c r="E188" s="15" t="n"/>
+      <c r="F188" s="15" t="n"/>
+      <c r="G188" s="15" t="n"/>
+      <c r="H188" s="15" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="111">
+  <mergeCells count="118">
     <mergeCell ref="A48:E48"/>
     <mergeCell ref="C142:E142"/>
     <mergeCell ref="C31:E31"/>
@@ -1760,6 +2158,7 @@
     <mergeCell ref="C140:E140"/>
     <mergeCell ref="C155:E155"/>
     <mergeCell ref="C18:E18"/>
+    <mergeCell ref="A5:H5"/>
     <mergeCell ref="C77:E77"/>
     <mergeCell ref="B101:E101"/>
     <mergeCell ref="A100:E100"/>
@@ -1777,6 +2176,7 @@
     <mergeCell ref="C168:E168"/>
     <mergeCell ref="B49:E49"/>
     <mergeCell ref="A157:E157"/>
+    <mergeCell ref="A186:H186"/>
     <mergeCell ref="C75:E75"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="C127:E127"/>
@@ -1788,6 +2188,7 @@
     <mergeCell ref="C169:E169"/>
     <mergeCell ref="B35:E35"/>
     <mergeCell ref="C52:E52"/>
+    <mergeCell ref="A187:H187"/>
     <mergeCell ref="C70:E70"/>
     <mergeCell ref="A133:E133"/>
     <mergeCell ref="C106:E106"/>
@@ -1795,6 +2196,7 @@
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="C161:E161"/>
     <mergeCell ref="C13:E13"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="B117:E117"/>
     <mergeCell ref="C15:E15"/>
@@ -1802,8 +2204,8 @@
     <mergeCell ref="B166:E166"/>
     <mergeCell ref="C79:E79"/>
     <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C121:E121"/>
     <mergeCell ref="C63:E63"/>
-    <mergeCell ref="C121:E121"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="B118:E118"/>
     <mergeCell ref="A24:E24"/>
@@ -1832,6 +2234,7 @@
     <mergeCell ref="B108:E108"/>
     <mergeCell ref="C137:E137"/>
     <mergeCell ref="C56:E56"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="C105:E105"/>
     <mergeCell ref="B85:E85"/>
     <mergeCell ref="C120:E120"/>
@@ -1849,8 +2252,10 @@
     <mergeCell ref="C102:E102"/>
     <mergeCell ref="C111:E111"/>
     <mergeCell ref="A116:E116"/>
+    <mergeCell ref="A185:H185"/>
     <mergeCell ref="C68:E68"/>
     <mergeCell ref="C58:E58"/>
+    <mergeCell ref="A184:H184"/>
     <mergeCell ref="B73:E73"/>
     <mergeCell ref="C97:E97"/>
     <mergeCell ref="C29:E29"/>
@@ -1951,5 +2356,14 @@
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;8 PECH Group Holdings Ltd | Confidential</oddHeader>
+    <oddFooter>&amp;C&amp;7 PECH Group Holdings Ltd | Lagos, Nigeria | pechgroupholdings.tech</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>